<commit_message>
feat(hero-caption): add contained variant; import prequalify, apply, dealer-tools
The dealer-tools hero (.subPageImageDealer) is a 1400px-wide combo photo
shown whole with the caption floating above the bottom edge; the parser
now emits hero-caption (contained) for it. Importer always uses the hero
image as the social image since the source og:image 404s.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,48 @@
     <t>url</t>
   </si>
   <si>
+    <t>apply.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>apply</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-10-11T04:53:42.316Z</t>
+  </si>
+  <si>
+    <t>Offer Buyers The Boat They Really Want With Easy Financing | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/apply/</t>
+  </si>
+  <si>
+    <t>dealer-tools.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","accordion-boxed","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>dealer-tools</t>
+  </si>
+  <si>
+    <t>2026-10-11T04:53:46.765Z</t>
+  </si>
+  <si>
+    <t>Access Useful Information For Getting Deals Done | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/dealer-tools/</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
@@ -46,9 +88,6 @@
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>home</t>
   </si>
   <si>
@@ -64,16 +103,10 @@
     <t>insurance.report.json</t>
   </si>
   <si>
-    <t>["hero-caption","columns-cta","columns-logos"]</t>
-  </si>
-  <si>
     <t>insurance</t>
   </si>
   <si>
-    <t>content-page</t>
-  </si>
-  <si>
-    <t>2026-10-11T03:03:40.170Z</t>
+    <t>2026-10-11T04:44:29.048Z</t>
   </si>
   <si>
     <t>Offer The Right Boat Insurance At The Right Price | Blue Water Finance</t>
@@ -88,7 +121,7 @@
     <t>loans</t>
   </si>
   <si>
-    <t>2026-10-11T03:03:30.822Z</t>
+    <t>2026-10-11T04:44:18.154Z</t>
   </si>
   <si>
     <t>Get More Deals Done With Expert Boat Financing | Blue Water Finance</t>
@@ -97,16 +130,28 @@
     <t>https://bluewaterfinance.com/loans/</t>
   </si>
   <si>
+    <t>prequalify.report.json</t>
+  </si>
+  <si>
+    <t>prequalify</t>
+  </si>
+  <si>
+    <t>2026-10-11T04:53:36.785Z</t>
+  </si>
+  <si>
+    <t>Find Out What Size Boat Your Customers Can Afford | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/prequalify/</t>
+  </si>
+  <si>
     <t>protection.report.json</t>
   </si>
   <si>
-    <t>["hero-caption","accordion-boxed","columns-cta","columns-logos"]</t>
-  </si>
-  <si>
     <t>protection</t>
   </si>
   <si>
-    <t>2026-10-11T03:03:36.348Z</t>
+    <t>2026-10-11T04:44:22.948Z</t>
   </si>
   <si>
     <t>Protect Your Customers With Leading Product Protection | Blue Water Finance</t>
@@ -501,16 +546,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="42" customWidth="1"/>
+    <col min="8" max="8" width="44" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -579,24 +624,24 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
@@ -605,24 +650,24 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
         <v>30</v>
@@ -631,7 +676,7 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
         <v>31</v>
@@ -641,6 +686,84 @@
       </c>
       <c r="H5" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(importer): link loan application forms to the source site
/prequalify/Application/, /apply/Application/ and /apply/co-applicant/ are
server-side credit applications (SSN, income, signatures) that stay on
bluewaterfinance.com; rewrite links to them as absolute source URLs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -52,7 +52,7 @@
     <t>content-page</t>
   </si>
   <si>
-    <t>2026-10-11T04:53:42.316Z</t>
+    <t>2026-10-11T05:28:55.682Z</t>
   </si>
   <si>
     <t>Offer Buyers The Boat They Really Want With Easy Financing | Blue Water Finance</t>
@@ -70,7 +70,7 @@
     <t>dealer-tools</t>
   </si>
   <si>
-    <t>2026-10-11T04:53:46.765Z</t>
+    <t>2026-10-11T05:29:00.404Z</t>
   </si>
   <si>
     <t>Access Useful Information For Getting Deals Done | Blue Water Finance</t>
@@ -91,7 +91,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-10-11T02:47:07.677Z</t>
+    <t>2026-10-11T05:28:49.075Z</t>
   </si>
   <si>
     <t>Blue Water Finance - Offering Superior Consumer Financing and Insurance services for Boat Dealers</t>
@@ -106,7 +106,7 @@
     <t>insurance</t>
   </si>
   <si>
-    <t>2026-10-11T04:44:29.048Z</t>
+    <t>2026-10-11T05:29:04.883Z</t>
   </si>
   <si>
     <t>Offer The Right Boat Insurance At The Right Price | Blue Water Finance</t>
@@ -121,7 +121,7 @@
     <t>loans</t>
   </si>
   <si>
-    <t>2026-10-11T04:44:18.154Z</t>
+    <t>2026-10-11T05:29:10.706Z</t>
   </si>
   <si>
     <t>Get More Deals Done With Expert Boat Financing | Blue Water Finance</t>
@@ -136,7 +136,7 @@
     <t>prequalify</t>
   </si>
   <si>
-    <t>2026-10-11T04:53:36.785Z</t>
+    <t>2026-10-11T05:29:15.738Z</t>
   </si>
   <si>
     <t>Find Out What Size Boat Your Customers Can Afford | Blue Water Finance</t>
@@ -151,7 +151,7 @@
     <t>protection</t>
   </si>
   <si>
-    <t>2026-10-11T04:44:22.948Z</t>
+    <t>2026-10-11T05:29:20.971Z</t>
   </si>
   <si>
     <t>Protect Your Customers With Leading Product Protection | Blue Water Finance</t>

</xml_diff>

<commit_message>
Add loan-calculator block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 15
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>_reportFile</t>
   </si>
@@ -158,6 +158,24 @@
   </si>
   <si>
     <t>https://bluewaterfinance.com/protection/</t>
+  </si>
+  <si>
+    <t>loans/loancalculator.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","loan-calculator","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>loans/loancalculator</t>
+  </si>
+  <si>
+    <t>2026-10-11T05:43:05.271Z</t>
+  </si>
+  <si>
+    <t>Calculate Loan Payments And Amounts | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/loans/LoanCalculator/</t>
   </si>
 </sst>
 </file>
@@ -546,16 +564,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -764,6 +781,32 @@
       </c>
       <c r="H8" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add cards-blog, form blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 113
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="92">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,21 +37,36 @@
     <t>url</t>
   </si>
   <si>
+    <t>about.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>content-page</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:28:32.640Z</t>
+  </si>
+  <si>
+    <t>About Us | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/about/</t>
+  </si>
+  <si>
     <t>apply.report.json</t>
   </si>
   <si>
-    <t>["hero-caption","columns-cta","columns-logos"]</t>
-  </si>
-  <si>
     <t>apply</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>content-page</t>
-  </si>
-  <si>
     <t>2026-10-11T05:28:55.682Z</t>
   </si>
   <si>
@@ -61,6 +76,42 @@
     <t>https://bluewaterfinance.com/apply/</t>
   </si>
   <si>
+    <t>blog.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","cards-blog","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>blog</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:28:45.547Z</t>
+  </si>
+  <si>
+    <t>Blog | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/blog/</t>
+  </si>
+  <si>
+    <t>contact.report.json</t>
+  </si>
+  <si>
+    <t>["hero-caption","form","columns-cta","columns-logos"]</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:28:39.084Z</t>
+  </si>
+  <si>
+    <t>Find Out How You Can Add Blue Water Finance To Your Dealership | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/contact/</t>
+  </si>
+  <si>
     <t>dealer-tools.report.json</t>
   </si>
   <si>
@@ -158,6 +209,66 @@
   </si>
   <si>
     <t>https://bluewaterfinance.com/protection/</t>
+  </si>
+  <si>
+    <t>blog/boat-insurance-why-offer-it-at-the-dealership.report.json</t>
+  </si>
+  <si>
+    <t>blog/boat-insurance-why-offer-it-at-the-dealership</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:28:54.717Z</t>
+  </si>
+  <si>
+    <t>Boat Insurance: Why Offer It at the Dealership? | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/blog/-boat-insurance-why-offer-it-at-the-dealership/</t>
+  </si>
+  <si>
+    <t>blog/helping-your-customers-navigate-boat-titling-a-guide-for-marine-dealers.report.json</t>
+  </si>
+  <si>
+    <t>blog/helping-your-customers-navigate-boat-titling-a-guide-for-marine-dealers</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:28:49.990Z</t>
+  </si>
+  <si>
+    <t>Helping Your Customers Navigate Boat Titling: A Guide for Marine Dealers | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/blog/helping-your-customers-navigate-boat-titling-a-guide-for-marine-dealers/</t>
+  </si>
+  <si>
+    <t>blog/maximize-success-during-boat-show-season.report.json</t>
+  </si>
+  <si>
+    <t>blog/maximize-success-during-boat-show-season</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:29:05.839Z</t>
+  </si>
+  <si>
+    <t>Maximize Success During Boat Show Season | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/blog/maximize-success-during-boat-show-season/</t>
+  </si>
+  <si>
+    <t>blog/unlocking-success-the-benefits-of-a-diverse-lender-portfolio.report.json</t>
+  </si>
+  <si>
+    <t>blog/unlocking-success-the-benefits-of-a-diverse-lender-portfolio</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:29:00.923Z</t>
+  </si>
+  <si>
+    <t>Unlocking Success: The Benefits of a Diverse Lender Portfolio | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/blog/unlocking-success-the-benefits-of-a-diverse-lender-portfolio/</t>
   </si>
   <si>
     <t>loans/loancalculator.report.json</t>
@@ -564,12 +675,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -632,85 +741,85 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -736,36 +845,36 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -774,24 +883,24 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -800,13 +909,195 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" t="s">
+        <v>69</v>
+      </c>
+      <c r="H12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H13" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>82</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>83</v>
+      </c>
+      <c r="G15" t="s">
+        <v>84</v>
+      </c>
+      <c r="H15" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>87</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add footer, header, loan-calculator blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 13
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-page.report.xlsx
+++ b/tools/importer/reports/import-content-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="107">
   <si>
     <t>_reportFile</t>
   </si>
@@ -209,6 +209,51 @@
   </si>
   <si>
     <t>https://bluewaterfinance.com/protection/</t>
+  </si>
+  <si>
+    <t>about/faq.report.json</t>
+  </si>
+  <si>
+    <t>about/faq</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:47:32.604Z</t>
+  </si>
+  <si>
+    <t>Frequently Asked Questions | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/about/faq/</t>
+  </si>
+  <si>
+    <t>about/protect-yourself-from-fraudulent-activity.report.json</t>
+  </si>
+  <si>
+    <t>about/protect-yourself-from-fraudulent-activity</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:47:37.903Z</t>
+  </si>
+  <si>
+    <t>Protect Yourself From Fraudulent Activity | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/about/protect-yourself-from-fraudulent-activity/</t>
+  </si>
+  <si>
+    <t>about/testimonials.report.json</t>
+  </si>
+  <si>
+    <t>about/testimonials</t>
+  </si>
+  <si>
+    <t>2026-10-11T15:47:26.920Z</t>
+  </si>
+  <si>
+    <t>Testimonials | Blue Water Finance</t>
+  </si>
+  <si>
+    <t>https://bluewaterfinance.com/about/testimonials/</t>
   </si>
   <si>
     <t>blog/boat-insurance-why-offer-it-at-the-dealership.report.json</t>
@@ -675,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1079,25 +1124,103 @@
         <v>86</v>
       </c>
       <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
         <v>87</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
         <v>88</v>
       </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>89</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>90</v>
       </c>
-      <c r="H16" t="s">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" t="s">
+        <v>94</v>
+      </c>
+      <c r="H17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" t="s">
+        <v>99</v>
+      </c>
+      <c r="H18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" t="s">
+        <v>105</v>
+      </c>
+      <c r="H19" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>